<commit_message>
Update: gitignore, kt.py, ma-thong-ke.xlsx
</commit_message>
<xml_diff>
--- a/ma-thong-ke.xlsx
+++ b/ma-thong-ke.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ketoan_doscom\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37C976B0-B25E-412C-8A9D-64B2AE92D52D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4922DE4F-0B7D-49D8-A878-696C5C378010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15840" xr2:uid="{C291A129-E5AA-4EFC-AA90-ED5132AA0EBC}"/>
   </bookViews>
@@ -355,7 +355,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -376,6 +376,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -694,6 +697,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECBED809-5768-4C04-9284-B08546E8EE0E}">
   <dimension ref="A1:C88"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="14.5703125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -1085,7 +1091,7 @@
       </c>
     </row>
     <row r="38" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="1">
+      <c r="A38" s="8">
         <v>641.1</v>
       </c>
       <c r="B38" s="4" t="s">
@@ -1096,7 +1102,7 @@
       </c>
     </row>
     <row r="39" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="1">
+      <c r="A39" s="8">
         <v>641.1</v>
       </c>
       <c r="B39" s="4" t="s">
@@ -1107,7 +1113,7 @@
       </c>
     </row>
     <row r="40" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="1">
+      <c r="A40" s="8">
         <v>641.1</v>
       </c>
       <c r="B40" s="4" t="s">
@@ -1118,7 +1124,7 @@
       </c>
     </row>
     <row r="41" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="1">
+      <c r="A41" s="8">
         <v>641.1</v>
       </c>
       <c r="B41" s="4" t="s">
@@ -1129,7 +1135,7 @@
       </c>
     </row>
     <row r="42" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="1">
+      <c r="A42" s="8">
         <v>641.1</v>
       </c>
       <c r="B42" s="5" t="s">
@@ -1431,7 +1437,7 @@
       </c>
     </row>
     <row r="70" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="1">
+      <c r="A70" s="8">
         <v>642.1</v>
       </c>
       <c r="B70" s="4" t="s">
@@ -1442,7 +1448,7 @@
       </c>
     </row>
     <row r="71" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="1">
+      <c r="A71" s="8">
         <v>642.1</v>
       </c>
       <c r="B71" s="4" t="s">
@@ -1453,7 +1459,7 @@
       </c>
     </row>
     <row r="72" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="1">
+      <c r="A72" s="8">
         <v>642.1</v>
       </c>
       <c r="B72" s="4" t="s">
@@ -1464,7 +1470,7 @@
       </c>
     </row>
     <row r="73" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="1">
+      <c r="A73" s="8">
         <v>642.1</v>
       </c>
       <c r="B73" s="4" t="s">
@@ -1475,7 +1481,7 @@
       </c>
     </row>
     <row r="74" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="1">
+      <c r="A74" s="8">
         <v>642.1</v>
       </c>
       <c r="B74" s="5" t="s">

</xml_diff>